<commit_message>
update proyectos desde streamlit
</commit_message>
<xml_diff>
--- a/proyectos_v2.xlsx
+++ b/proyectos_v2.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="proyectos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stock_dispo" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lavado" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="proyectos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="stock_dispo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="lavado" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,16 +22,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -50,21 +47,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -435,82 +423,82 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Constructora</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Fecha_requerida</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>M2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Avance_pct</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Avance_m2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Ritmo_esperado</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Inicio_obra</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Duracion_obra_meses</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Termino_obra</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>WF600x2250_usado</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>WF600x2250_nuevo</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>CE600x1200_usado</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>CE600x1200_nuevo</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Comentario</t>
         </is>
@@ -532,7 +520,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="1" t="n">
         <v>46073</v>
       </c>
       <c r="E2" t="n">
@@ -545,13 +533,13 @@
         <v>1200</v>
       </c>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" s="2" t="n">
+      <c r="I2" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="J2" t="n">
         <v>5</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="K2" s="1" t="n">
         <v>46200</v>
       </c>
       <c r="L2" t="n">
@@ -584,7 +572,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="1" t="n">
         <v>46074</v>
       </c>
       <c r="E3" t="n">
@@ -597,13 +585,13 @@
         <v>812</v>
       </c>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" s="2" t="n">
+      <c r="I3" s="1" t="n">
         <v>46074</v>
       </c>
       <c r="J3" t="n">
         <v>3.2</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="K3" s="1" t="n">
         <v>46170</v>
       </c>
       <c r="L3" t="n">
@@ -636,7 +624,7 @@
           <t>Arriendo</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="1" t="n">
         <v>46070</v>
       </c>
       <c r="E4" t="n">
@@ -649,13 +637,13 @@
         <v>300</v>
       </c>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" s="2" t="n">
+      <c r="I4" s="1" t="n">
         <v>46052</v>
       </c>
       <c r="J4" t="n">
         <v>1.5</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="K4" s="1" t="n">
         <v>46097</v>
       </c>
       <c r="L4" t="n">
@@ -688,7 +676,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="E5" t="n">
@@ -701,13 +689,13 @@
         <v>834</v>
       </c>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" s="2" t="n">
+      <c r="I5" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="J5" t="n">
         <v>7</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="1" t="n">
         <v>46330</v>
       </c>
       <c r="L5" t="n">
@@ -740,7 +728,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="E6" t="n">
@@ -753,13 +741,13 @@
         <v>100</v>
       </c>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" s="2" t="n">
+      <c r="I6" s="1" t="n">
         <v>46008</v>
       </c>
       <c r="J6" t="n">
         <v>4</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="K6" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="L6" t="n">
@@ -788,7 +776,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="1" t="n">
         <v>46118</v>
       </c>
       <c r="E7" t="n">
@@ -801,13 +789,13 @@
         <v>812</v>
       </c>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" s="2" t="n">
+      <c r="I7" s="1" t="n">
         <v>46118</v>
       </c>
       <c r="J7" t="n">
         <v>6</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="K7" s="1" t="n">
         <v>46298</v>
       </c>
       <c r="L7" t="n">
@@ -838,26 +826,26 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="1" t="n">
         <v>46150</v>
       </c>
       <c r="E8" t="n">
         <v>353</v>
       </c>
       <c r="F8" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>335.35</v>
+        <v>353</v>
       </c>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" s="2" t="n">
+      <c r="I8" s="1" t="n">
         <v>46150</v>
       </c>
       <c r="J8" t="n">
         <v>6</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="K8" s="1" t="n">
         <v>46330</v>
       </c>
       <c r="L8" t="n">
@@ -886,7 +874,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" s="1" t="n">
         <v>46090</v>
       </c>
       <c r="E9" t="n">
@@ -899,13 +887,13 @@
         <v>511</v>
       </c>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" s="2" t="n">
+      <c r="I9" s="1" t="n">
         <v>46090</v>
       </c>
       <c r="J9" t="n">
         <v>5</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="K9" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="L9" t="n">
@@ -934,7 +922,7 @@
           <t>Arriendo</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" s="1" t="n">
         <v>46022</v>
       </c>
       <c r="E10" t="n">
@@ -947,13 +935,13 @@
         <v>300</v>
       </c>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" s="2" t="n">
+      <c r="I10" s="1" t="n">
         <v>46022</v>
       </c>
       <c r="J10" t="n">
         <v>2</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="K10" s="1" t="n">
         <v>46082</v>
       </c>
       <c r="L10" t="n">
@@ -982,7 +970,7 @@
           <t>Arriendo</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="1" t="n">
         <v>45888</v>
       </c>
       <c r="E11" t="n">
@@ -995,13 +983,13 @@
         <v>0</v>
       </c>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" s="2" t="n">
+      <c r="I11" s="1" t="n">
         <v>45888</v>
       </c>
       <c r="J11" t="n">
         <v>12</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="K11" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="L11" t="n">
@@ -1030,7 +1018,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="E12" t="n">
@@ -1043,13 +1031,13 @@
         <v>653</v>
       </c>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" s="2" t="n">
+      <c r="I12" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="J12" t="n">
         <v>5</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="K12" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="L12" t="n">
@@ -1080,7 +1068,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D13" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="E13" t="n">
@@ -1093,13 +1081,13 @@
         <v>0</v>
       </c>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" s="2" t="n">
+      <c r="I13" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="J13" t="n">
         <v>3</v>
       </c>
-      <c r="K13" s="2" t="n">
+      <c r="K13" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="L13" t="n">
@@ -1132,7 +1120,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="E14" t="n">
@@ -1145,13 +1133,13 @@
         <v>381</v>
       </c>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" s="2" t="n">
+      <c r="I14" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="J14" t="n">
         <v>3</v>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="K14" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="L14" t="n">
@@ -1180,7 +1168,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D15" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="E15" t="n">
@@ -1193,13 +1181,13 @@
         <v>0</v>
       </c>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" s="2" t="n">
+      <c r="I15" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="J15" t="n">
         <v>5</v>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="K15" s="1" t="n">
         <v>46359</v>
       </c>
       <c r="L15" t="n">
@@ -1232,7 +1220,7 @@
           <t>Venta</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D16" s="1" t="n">
         <v>46081</v>
       </c>
       <c r="E16" t="n">
@@ -1247,7 +1235,7 @@
       <c r="H16" t="n">
         <v>5</v>
       </c>
-      <c r="I16" s="2" t="n">
+      <c r="I16" s="1" t="n">
         <v>46081</v>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -1274,7 +1262,7 @@
           <t>Venta</t>
         </is>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="D17" s="1" t="n">
         <v>46087</v>
       </c>
       <c r="E17" t="n">
@@ -1289,7 +1277,7 @@
       <c r="H17" t="n">
         <v>5</v>
       </c>
-      <c r="I17" s="2" t="n">
+      <c r="I17" s="1" t="n">
         <v>46087</v>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1316,7 +1304,7 @@
           <t>Venta</t>
         </is>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D18" s="1" t="n">
         <v>46151</v>
       </c>
       <c r="E18" t="n">
@@ -1329,7 +1317,7 @@
         <v>0</v>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" s="2" t="n">
+      <c r="I18" s="1" t="n">
         <v>46151</v>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1356,7 +1344,7 @@
           <t>Reparación</t>
         </is>
       </c>
-      <c r="D19" s="2" t="n">
+      <c r="D19" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="E19" t="n">
@@ -1369,7 +1357,7 @@
         <v>500</v>
       </c>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" s="2" t="n">
+      <c r="I19" s="1" t="n">
         <v>46127</v>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -1396,7 +1384,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D20" s="2" t="n">
+      <c r="D20" s="1" t="n">
         <v>45901</v>
       </c>
       <c r="E20" t="n">
@@ -1409,13 +1397,13 @@
         <v>0</v>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" s="2" t="n">
+      <c r="I20" s="1" t="n">
         <v>45901</v>
       </c>
       <c r="J20" t="n">
         <v>6.5</v>
       </c>
-      <c r="K20" s="2" t="n">
+      <c r="K20" s="1" t="n">
         <v>46096</v>
       </c>
       <c r="L20" t="n">
@@ -1444,7 +1432,7 @@
           <t>Venta</t>
         </is>
       </c>
-      <c r="D21" s="2" t="n">
+      <c r="D21" s="1" t="n">
         <v>46002</v>
       </c>
       <c r="E21" t="n">
@@ -1457,7 +1445,7 @@
         <v>0</v>
       </c>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" s="2" t="n">
+      <c r="I21" s="1" t="n">
         <v>46002</v>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -1488,7 +1476,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D22" s="2" t="n">
+      <c r="D22" s="1" t="n">
         <v>46023</v>
       </c>
       <c r="E22" t="n">
@@ -1501,13 +1489,13 @@
         <v>0</v>
       </c>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" s="2" t="n">
+      <c r="I22" s="1" t="n">
         <v>46023</v>
       </c>
       <c r="J22" t="n">
         <v>1.5</v>
       </c>
-      <c r="K22" s="2" t="n">
+      <c r="K22" s="1" t="n">
         <v>46068</v>
       </c>
       <c r="L22" t="n">
@@ -1536,7 +1524,7 @@
           <t>Venta</t>
         </is>
       </c>
-      <c r="D23" s="2" t="n">
+      <c r="D23" s="1" t="n">
         <v>46041</v>
       </c>
       <c r="E23" t="n">
@@ -1549,7 +1537,7 @@
         <v>0</v>
       </c>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" s="2" t="n">
+      <c r="I23" s="1" t="n">
         <v>46041</v>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -1578,7 +1566,7 @@
           <t>Venta</t>
         </is>
       </c>
-      <c r="D24" s="2" t="n">
+      <c r="D24" s="1" t="n">
         <v>46041</v>
       </c>
       <c r="E24" t="n">
@@ -1591,7 +1579,7 @@
         <v>0</v>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="I24" s="2" t="n">
+      <c r="I24" s="1" t="n">
         <v>46041</v>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -1620,7 +1608,7 @@
           <t>Reparación</t>
         </is>
       </c>
-      <c r="D25" s="2" t="n">
+      <c r="D25" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="E25" t="n">
@@ -1633,7 +1621,7 @@
         <v>855</v>
       </c>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" s="2" t="n">
+      <c r="I25" s="1" t="n">
         <v>46104</v>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -1660,7 +1648,7 @@
           <t>Reparación</t>
         </is>
       </c>
-      <c r="D26" s="2" t="n">
+      <c r="D26" s="1" t="n">
         <v>46179</v>
       </c>
       <c r="E26" t="n">
@@ -1673,7 +1661,7 @@
         <v>0</v>
       </c>
       <c r="H26" t="inlineStr"/>
-      <c r="I26" s="2" t="n">
+      <c r="I26" s="1" t="n">
         <v>46178</v>
       </c>
       <c r="J26" t="inlineStr"/>
@@ -1700,7 +1688,7 @@
           <t>Arriendo</t>
         </is>
       </c>
-      <c r="D27" s="2" t="n">
+      <c r="D27" s="1" t="n">
         <v>46092</v>
       </c>
       <c r="E27" t="n">
@@ -1713,7 +1701,7 @@
         <v>27.6</v>
       </c>
       <c r="H27" t="inlineStr"/>
-      <c r="I27" s="2" t="n">
+      <c r="I27" s="1" t="n">
         <v>46092</v>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -1740,7 +1728,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D28" s="2" t="n">
+      <c r="D28" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="E28" t="n">
@@ -1753,7 +1741,7 @@
         <v>0</v>
       </c>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" s="2" t="n">
+      <c r="I28" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="J28" t="inlineStr"/>
@@ -1780,7 +1768,7 @@
           <t>Venta</t>
         </is>
       </c>
-      <c r="D29" s="2" t="n">
+      <c r="D29" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="E29" t="n">
@@ -1793,7 +1781,7 @@
         <v>0</v>
       </c>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" s="2" t="n">
+      <c r="I29" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -1824,7 +1812,7 @@
           <t>Reparación</t>
         </is>
       </c>
-      <c r="D30" s="2" t="n">
+      <c r="D30" s="1" t="n">
         <v>46129</v>
       </c>
       <c r="E30" t="n">
@@ -1837,7 +1825,7 @@
         <v>230</v>
       </c>
       <c r="H30" t="inlineStr"/>
-      <c r="I30" s="2" t="n">
+      <c r="I30" s="1" t="n">
         <v>46129</v>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -1868,7 +1856,7 @@
           <t>Reparación</t>
         </is>
       </c>
-      <c r="D31" s="2" t="n">
+      <c r="D31" s="1" t="n">
         <v>46151</v>
       </c>
       <c r="E31" t="n">
@@ -1881,7 +1869,7 @@
         <v>0</v>
       </c>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" s="2" t="n">
+      <c r="I31" s="1" t="n">
         <v>46151</v>
       </c>
       <c r="J31" t="inlineStr"/>
@@ -1908,7 +1896,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D32" s="2" t="n">
+      <c r="D32" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="E32" t="n">
@@ -1921,13 +1909,13 @@
         <v>0</v>
       </c>
       <c r="H32" t="inlineStr"/>
-      <c r="I32" s="2" t="n">
+      <c r="I32" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="J32" t="n">
         <v>3.5</v>
       </c>
-      <c r="K32" s="2" t="n">
+      <c r="K32" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="L32" t="n">
@@ -1956,7 +1944,7 @@
           <t>Venta</t>
         </is>
       </c>
-      <c r="D33" s="2" t="n">
+      <c r="D33" s="1" t="n">
         <v>46108</v>
       </c>
       <c r="E33" t="n">
@@ -1971,7 +1959,7 @@
       <c r="H33" t="n">
         <v>5</v>
       </c>
-      <c r="I33" s="2" t="n">
+      <c r="I33" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="J33" t="inlineStr"/>
@@ -1998,7 +1986,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D34" s="2" t="n">
+      <c r="D34" s="1" t="n">
         <v>46181</v>
       </c>
       <c r="E34" t="n">
@@ -2011,13 +1999,13 @@
         <v>0</v>
       </c>
       <c r="H34" t="inlineStr"/>
-      <c r="I34" s="2" t="n">
+      <c r="I34" s="1" t="n">
         <v>46181</v>
       </c>
       <c r="J34" t="n">
         <v>9</v>
       </c>
-      <c r="K34" s="2" t="n">
+      <c r="K34" s="1" t="n">
         <v>46451</v>
       </c>
       <c r="L34" t="n">
@@ -2054,7 +2042,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D35" s="2" t="n">
+      <c r="D35" s="1" t="n">
         <v>46195</v>
       </c>
       <c r="E35" t="n">
@@ -2067,13 +2055,13 @@
         <v>0</v>
       </c>
       <c r="H35" t="inlineStr"/>
-      <c r="I35" s="2" t="n">
+      <c r="I35" s="1" t="n">
         <v>46195</v>
       </c>
       <c r="J35" t="n">
         <v>3</v>
       </c>
-      <c r="K35" s="2" t="n">
+      <c r="K35" s="1" t="n">
         <v>46285</v>
       </c>
       <c r="L35" t="n">
@@ -2110,7 +2098,7 @@
           <t>Venta</t>
         </is>
       </c>
-      <c r="D36" s="2" t="n">
+      <c r="D36" s="1" t="n">
         <v>46154</v>
       </c>
       <c r="E36" t="n">
@@ -2123,7 +2111,7 @@
         <v>40</v>
       </c>
       <c r="H36" t="inlineStr"/>
-      <c r="I36" s="2" t="n">
+      <c r="I36" s="1" t="n">
         <v>46154</v>
       </c>
       <c r="J36" t="inlineStr"/>
@@ -2150,7 +2138,7 @@
           <t>Venta</t>
         </is>
       </c>
-      <c r="D37" s="2" t="n">
+      <c r="D37" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="E37" t="n">
@@ -2163,7 +2151,7 @@
         <v>0</v>
       </c>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" s="2" t="n">
+      <c r="I37" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="J37" t="inlineStr"/>
@@ -2198,7 +2186,7 @@
           <t>Venta</t>
         </is>
       </c>
-      <c r="D38" s="2" t="n">
+      <c r="D38" s="1" t="n">
         <v>46220</v>
       </c>
       <c r="E38" t="n">
@@ -2211,7 +2199,7 @@
         <v>0</v>
       </c>
       <c r="H38" t="inlineStr"/>
-      <c r="I38" s="2" t="n">
+      <c r="I38" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="J38" t="inlineStr"/>
@@ -2242,7 +2230,7 @@
           <t>Arriendo MO</t>
         </is>
       </c>
-      <c r="D39" s="2" t="n">
+      <c r="D39" s="1" t="n">
         <v>46230</v>
       </c>
       <c r="E39" t="n">
@@ -2255,7 +2243,7 @@
         <v>0</v>
       </c>
       <c r="H39" t="inlineStr"/>
-      <c r="I39" s="2" t="n">
+      <c r="I39" s="1" t="n">
         <v>46230</v>
       </c>
       <c r="J39" t="inlineStr"/>
@@ -2282,7 +2270,7 @@
           <t>Reparación</t>
         </is>
       </c>
-      <c r="D40" s="2" t="n">
+      <c r="D40" s="1" t="n">
         <v>46195</v>
       </c>
       <c r="E40" t="n">
@@ -2295,7 +2283,7 @@
         <v>0</v>
       </c>
       <c r="H40" t="inlineStr"/>
-      <c r="I40" s="2" t="n">
+      <c r="I40" s="1" t="n">
         <v>46195</v>
       </c>
       <c r="J40" t="inlineStr"/>
@@ -2322,7 +2310,7 @@
           <t>Venta</t>
         </is>
       </c>
-      <c r="D41" s="2" t="n">
+      <c r="D41" s="1" t="n">
         <v>46175</v>
       </c>
       <c r="E41" t="n">
@@ -2335,7 +2323,7 @@
         <v>0</v>
       </c>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" s="2" t="n">
+      <c r="I41" s="1" t="n">
         <v>46197</v>
       </c>
       <c r="J41" t="inlineStr"/>
@@ -2362,7 +2350,7 @@
           <t>Arriendo</t>
         </is>
       </c>
-      <c r="D42" s="2" t="n">
+      <c r="D42" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="E42" t="n">
@@ -2375,13 +2363,13 @@
         <v>0</v>
       </c>
       <c r="H42" t="inlineStr"/>
-      <c r="I42" s="2" t="n">
+      <c r="I42" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="J42" t="n">
         <v>6.5</v>
       </c>
-      <c r="K42" s="2" t="n">
+      <c r="K42" s="1" t="n">
         <v>46461</v>
       </c>
       <c r="L42" t="inlineStr"/>
@@ -2401,43 +2389,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>WF600x2250_nuevo</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>WF600x2250_usado</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>CE600x1200_nuevo</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>CE600x1200_usado</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Comentario</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>45901</v>
       </c>
       <c r="B2" t="n">
@@ -2459,7 +2447,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>46095</v>
       </c>
       <c r="B3" t="n">
@@ -2477,7 +2465,7 @@
       <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="B4" t="n">
@@ -2495,7 +2483,7 @@
       <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="B5" t="n">
@@ -2511,6 +2499,22 @@
         <v>0</v>
       </c>
       <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2527,57 +2531,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Constructora</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>M2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Avance</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Inicio</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Termino</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Fecha Requerida</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Ritmo</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Holgura</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Inicio_prog</t>
         </is>
@@ -2602,7 +2606,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="1" t="n">
         <v>45996</v>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -2629,7 +2633,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -2656,7 +2660,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="1" t="n">
         <v>46048</v>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -2683,7 +2687,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" s="2" t="n">
+      <c r="G5" s="1" t="n">
         <v>46069</v>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -2710,7 +2714,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" s="2" t="n">
+      <c r="G6" s="1" t="n">
         <v>46066</v>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -2737,7 +2741,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="1" t="n">
         <v>46035</v>
       </c>
       <c r="H7" t="inlineStr"/>

</xml_diff>

<commit_message>
autosave proyectos desde streamlit
</commit_message>
<xml_diff>
--- a/proyectos_v2.xlsx
+++ b/proyectos_v2.xlsx
@@ -1075,10 +1075,10 @@
         <v>500</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" s="1" t="n">

</xml_diff>

<commit_message>
edición: update automático desde streamlit
</commit_message>
<xml_diff>
--- a/proyectos_v2.xlsx
+++ b/proyectos_v2.xlsx
@@ -1311,10 +1311,10 @@
         <v>276</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>55.2</v>
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" s="1" t="n">

</xml_diff>

<commit_message>
Actualización de datos desde Streamlit
</commit_message>
<xml_diff>
--- a/proyectos_v2.xlsx
+++ b/proyectos_v2.xlsx
@@ -1903,10 +1903,10 @@
         <v>430</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="H32" t="inlineStr"/>
       <c r="I32" s="1" t="n">

</xml_diff>